<commit_message>
feat: implement product color variations and interactive UI swatches across all pages
</commit_message>
<xml_diff>
--- a/src/assets/data.xlsx
+++ b/src/assets/data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TVH01374\Downloads\img\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TUF\Desktop\tamdoor\src\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2B3CC2D-6805-40EE-830E-DFD811A37B3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2836BD82-4FD7-4C18-A4CB-EF6FBEBF4DBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{9ED37A15-96E1-4502-9623-4C4A39A8DE50}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{9ED37A15-96E1-4502-9623-4C4A39A8DE50}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="37">
   <si>
     <t>Tên sản phẩm</t>
   </si>
@@ -138,6 +138,15 @@
   </si>
   <si>
     <t>khoa-hafele.jpg</t>
+  </si>
+  <si>
+    <t>Vân gỗ Sồi:soi.jpg;Óc chó:occho.jpg;Trắng sứ:trang.jpg</t>
+  </si>
+  <si>
+    <t>Màu Sắc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Vàng nhạt:vang.png;Xám đậm:xam.png</t>
   </si>
 </sst>
 </file>
@@ -209,7 +218,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -223,9 +232,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1" readingOrder="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -241,7 +253,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Chủ đề Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -557,7 +569,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F94A27B-426F-4566-8D8A-C84BD576F6F8}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="30.875" customWidth="1"/>
@@ -568,9 +580,10 @@
     <col min="6" max="6" width="20.375" customWidth="1"/>
     <col min="7" max="7" width="40.5" customWidth="1"/>
     <col min="8" max="8" width="53.75" customWidth="1"/>
+    <col min="9" max="9" width="48.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="36.75" customHeight="1" thickBot="1">
+    <row r="1" spans="1:9" ht="36.75" customHeight="1" thickBot="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -595,8 +608,11 @@
       <c r="H1" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>35</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" ht="29.25" thickBot="1">
+    <row r="2" spans="1:9" ht="29.25" thickBot="1">
       <c r="A2" s="2" t="s">
         <v>13</v>
       </c>
@@ -621,8 +637,11 @@
       <c r="H2" s="2" t="s">
         <v>17</v>
       </c>
+      <c r="I2" s="5" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="3" spans="1:8" ht="29.25" thickBot="1">
+    <row r="3" spans="1:9" ht="29.25" thickBot="1">
       <c r="A3" s="2" t="s">
         <v>18</v>
       </c>
@@ -647,8 +666,11 @@
       <c r="H3" s="2" t="s">
         <v>21</v>
       </c>
+      <c r="I3" t="s">
+        <v>36</v>
+      </c>
     </row>
-    <row r="4" spans="1:8" ht="37.5" customHeight="1" thickBot="1">
+    <row r="4" spans="1:9" ht="37.5" customHeight="1" thickBot="1">
       <c r="A4" s="2" t="s">
         <v>22</v>
       </c>
@@ -673,8 +695,9 @@
       <c r="H4" s="2" t="s">
         <v>27</v>
       </c>
+      <c r="I4" s="2"/>
     </row>
-    <row r="5" spans="1:8" ht="29.25" thickBot="1">
+    <row r="5" spans="1:9" ht="29.25" thickBot="1">
       <c r="A5" s="2" t="s">
         <v>28</v>
       </c>
@@ -699,6 +722,7 @@
       <c r="H5" s="2" t="s">
         <v>32</v>
       </c>
+      <c r="I5" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>